<commit_message>
Enlace para firmas de operarios, una vez firmado, se redirige al logoout. ocultado boton de actualizar matriz de polivalencia, solo se puede editar, no actualizar desde la app.
</commit_message>
<xml_diff>
--- a/TPL-708 [4] RCSE Matriz de Polivalencia Operarios producción.xlsx
+++ b/TPL-708 [4] RCSE Matriz de Polivalencia Operarios producción.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29728C03-7284-468D-99EF-CF87F4200216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E72004-E140-4EC7-B247-8BCE7D8EA577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45120" yWindow="-8490" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{99D3D415-75B1-45FF-A9DD-36F70A54E67C}"/>
+    <workbookView xWindow="-45105" yWindow="150" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{99D3D415-75B1-45FF-A9DD-36F70A54E67C}"/>
   </bookViews>
   <sheets>
     <sheet name="Operarios producción V1.00" sheetId="2" state="hidden" r:id="rId1"/>
@@ -1500,7 +1500,7 @@
     <t>EDUARDO PAREDES</t>
   </si>
   <si>
-    <t>RPM-Decontaminación</t>
+    <t>RPM-Descontaminación</t>
   </si>
 </sst>
 </file>
@@ -10186,7 +10186,7 @@
       <c r="AX2" s="36"/>
       <c r="AY2" s="36"/>
     </row>
-    <row r="3" spans="1:51" ht="156.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:51" ht="139" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="18" t="s">
         <v>0</v>
       </c>
@@ -10341,7 +10341,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="4" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>209</v>
       </c>
@@ -10483,7 +10483,7 @@
       <c r="AX5" s="3"/>
       <c r="AY5" s="3"/>
     </row>
-    <row r="6" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
         <v>399</v>
       </c>
@@ -10540,7 +10540,7 @@
       <c r="AX6" s="3"/>
       <c r="AY6" s="3"/>
     </row>
-    <row r="7" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
         <v>425</v>
       </c>
@@ -10597,7 +10597,7 @@
       <c r="AX7" s="3"/>
       <c r="AY7" s="3"/>
     </row>
-    <row r="8" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
         <v>439</v>
       </c>
@@ -10654,7 +10654,7 @@
       <c r="AX8" s="3"/>
       <c r="AY8" s="3"/>
     </row>
-    <row r="9" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>210</v>
       </c>
@@ -10833,7 +10833,7 @@
       <c r="AX11" s="3"/>
       <c r="AY11" s="3"/>
     </row>
-    <row r="12" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
         <v>213</v>
       </c>
@@ -10963,7 +10963,7 @@
       <c r="AX13" s="3"/>
       <c r="AY13" s="3"/>
     </row>
-    <row r="14" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
         <v>383</v>
       </c>
@@ -11020,7 +11020,7 @@
       <c r="AX14" s="3"/>
       <c r="AY14" s="3"/>
     </row>
-    <row r="15" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
         <v>402</v>
       </c>
@@ -11081,7 +11081,7 @@
       <c r="AX15" s="3"/>
       <c r="AY15" s="3"/>
     </row>
-    <row r="16" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
         <v>215</v>
       </c>
@@ -11138,7 +11138,7 @@
       <c r="AX16" s="3"/>
       <c r="AY16" s="3"/>
     </row>
-    <row r="17" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="23" t="s">
         <v>34</v>
       </c>
@@ -11213,7 +11213,7 @@
       <c r="AX17" s="3"/>
       <c r="AY17" s="3"/>
     </row>
-    <row r="18" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
         <v>216</v>
       </c>
@@ -11276,7 +11276,7 @@
       <c r="AX18" s="3"/>
       <c r="AY18" s="3"/>
     </row>
-    <row r="19" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="23" t="s">
         <v>460</v>
       </c>
@@ -11335,7 +11335,7 @@
       <c r="AX19" s="3"/>
       <c r="AY19" s="3"/>
     </row>
-    <row r="20" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A20" s="23" t="s">
         <v>217</v>
       </c>
@@ -11455,7 +11455,7 @@
       <c r="AX21" s="3"/>
       <c r="AY21" s="3"/>
     </row>
-    <row r="22" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A22" s="23" t="s">
         <v>37</v>
       </c>
@@ -11524,7 +11524,7 @@
       <c r="AX22" s="3"/>
       <c r="AY22" s="3"/>
     </row>
-    <row r="23" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
         <v>220</v>
       </c>
@@ -11585,7 +11585,7 @@
       <c r="AX23" s="3"/>
       <c r="AY23" s="3"/>
     </row>
-    <row r="24" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A24" s="23" t="s">
         <v>426</v>
       </c>
@@ -11642,7 +11642,7 @@
       <c r="AX24" s="3"/>
       <c r="AY24" s="3"/>
     </row>
-    <row r="25" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
         <v>221</v>
       </c>
@@ -11699,7 +11699,7 @@
       <c r="AX25" s="3"/>
       <c r="AY25" s="3"/>
     </row>
-    <row r="26" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A26" s="23" t="s">
         <v>38</v>
       </c>
@@ -11762,7 +11762,7 @@
       <c r="AX26" s="3"/>
       <c r="AY26" s="3"/>
     </row>
-    <row r="27" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A27" s="23" t="s">
         <v>222</v>
       </c>
@@ -11819,7 +11819,7 @@
       <c r="AX27" s="3"/>
       <c r="AY27" s="3"/>
     </row>
-    <row r="28" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A28" s="23" t="s">
         <v>223</v>
       </c>
@@ -11878,7 +11878,7 @@
       <c r="AX28" s="3"/>
       <c r="AY28" s="3"/>
     </row>
-    <row r="29" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A29" s="23" t="s">
         <v>224</v>
       </c>
@@ -11941,7 +11941,7 @@
       <c r="AX29" s="3"/>
       <c r="AY29" s="3"/>
     </row>
-    <row r="30" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
         <v>443</v>
       </c>
@@ -12000,7 +12000,7 @@
       <c r="AX30" s="3"/>
       <c r="AY30" s="3"/>
     </row>
-    <row r="31" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>225</v>
       </c>
@@ -12061,7 +12061,7 @@
       <c r="AX31" s="3"/>
       <c r="AY31" s="3"/>
     </row>
-    <row r="32" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
         <v>226</v>
       </c>
@@ -12120,7 +12120,7 @@
       <c r="AX32" s="3"/>
       <c r="AY32" s="3"/>
     </row>
-    <row r="33" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A33" s="23" t="s">
         <v>44</v>
       </c>
@@ -12189,7 +12189,7 @@
       <c r="AX33" s="3"/>
       <c r="AY33" s="3"/>
     </row>
-    <row r="34" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A34" s="23" t="s">
         <v>227</v>
       </c>
@@ -12307,7 +12307,7 @@
       <c r="AX35" s="3"/>
       <c r="AY35" s="3"/>
     </row>
-    <row r="36" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A36" s="23" t="s">
         <v>452</v>
       </c>
@@ -12425,7 +12425,7 @@
       <c r="AX37" s="3"/>
       <c r="AY37" s="3"/>
     </row>
-    <row r="38" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A38" s="23" t="s">
         <v>230</v>
       </c>
@@ -12545,7 +12545,7 @@
       <c r="AX39" s="3"/>
       <c r="AY39" s="3"/>
     </row>
-    <row r="40" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A40" s="23" t="s">
         <v>48</v>
       </c>
@@ -12612,7 +12612,7 @@
       <c r="AX40" s="3"/>
       <c r="AY40" s="3"/>
     </row>
-    <row r="41" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A41" s="23" t="s">
         <v>375</v>
       </c>
@@ -12669,7 +12669,7 @@
       <c r="AX41" s="3"/>
       <c r="AY41" s="3"/>
     </row>
-    <row r="42" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A42" s="23" t="s">
         <v>435</v>
       </c>
@@ -12726,7 +12726,7 @@
       <c r="AX42" s="3"/>
       <c r="AY42" s="3"/>
     </row>
-    <row r="43" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A43" s="23" t="s">
         <v>231</v>
       </c>
@@ -12789,7 +12789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A44" s="23" t="s">
         <v>49</v>
       </c>
@@ -12862,7 +12862,7 @@
       <c r="AX44" s="3"/>
       <c r="AY44" s="3"/>
     </row>
-    <row r="45" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A45" s="23" t="s">
         <v>50</v>
       </c>
@@ -12929,7 +12929,7 @@
       <c r="AX45" s="3"/>
       <c r="AY45" s="3"/>
     </row>
-    <row r="46" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A46" s="23" t="s">
         <v>232</v>
       </c>
@@ -12988,7 +12988,7 @@
       <c r="AX46" s="3"/>
       <c r="AY46" s="3"/>
     </row>
-    <row r="47" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A47" s="23" t="s">
         <v>431</v>
       </c>
@@ -13112,7 +13112,7 @@
       <c r="AX48" s="3"/>
       <c r="AY48" s="3"/>
     </row>
-    <row r="49" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A49" s="23" t="s">
         <v>234</v>
       </c>
@@ -13177,7 +13177,7 @@
       <c r="AX49" s="3"/>
       <c r="AY49" s="3"/>
     </row>
-    <row r="50" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A50" s="23" t="s">
         <v>51</v>
       </c>
@@ -13250,7 +13250,7 @@
       <c r="AX50" s="3"/>
       <c r="AY50" s="3"/>
     </row>
-    <row r="51" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A51" s="23" t="s">
         <v>438</v>
       </c>
@@ -13307,7 +13307,7 @@
       <c r="AX51" s="3"/>
       <c r="AY51" s="3"/>
     </row>
-    <row r="52" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A52" s="23" t="s">
         <v>52</v>
       </c>
@@ -13368,7 +13368,7 @@
       <c r="AX52" s="3"/>
       <c r="AY52" s="3"/>
     </row>
-    <row r="53" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A53" s="23" t="s">
         <v>235</v>
       </c>
@@ -13427,7 +13427,7 @@
       <c r="AX53" s="3"/>
       <c r="AY53" s="3"/>
     </row>
-    <row r="54" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A54" s="23" t="s">
         <v>53</v>
       </c>
@@ -13494,7 +13494,7 @@
       <c r="AX54" s="3"/>
       <c r="AY54" s="3"/>
     </row>
-    <row r="55" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A55" s="23" t="s">
         <v>236</v>
       </c>
@@ -13551,7 +13551,7 @@
       <c r="AX55" s="3"/>
       <c r="AY55" s="3"/>
     </row>
-    <row r="56" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A56" s="23" t="s">
         <v>54</v>
       </c>
@@ -13620,7 +13620,7 @@
       <c r="AX56" s="3"/>
       <c r="AY56" s="3"/>
     </row>
-    <row r="57" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A57" s="23" t="s">
         <v>414</v>
       </c>
@@ -13799,7 +13799,7 @@
       <c r="AX59" s="3"/>
       <c r="AY59" s="3"/>
     </row>
-    <row r="60" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A60" s="23" t="s">
         <v>57</v>
       </c>
@@ -13862,7 +13862,7 @@
       <c r="AX60" s="3"/>
       <c r="AY60" s="3"/>
     </row>
-    <row r="61" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A61" s="23" t="s">
         <v>58</v>
       </c>
@@ -13929,7 +13929,7 @@
       <c r="AX61" s="3"/>
       <c r="AY61" s="3"/>
     </row>
-    <row r="62" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A62" s="23" t="s">
         <v>239</v>
       </c>
@@ -13998,7 +13998,7 @@
       <c r="AX62" s="3"/>
       <c r="AY62" s="3"/>
     </row>
-    <row r="63" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A63" s="23" t="s">
         <v>240</v>
       </c>
@@ -14065,7 +14065,7 @@
       <c r="AX63" s="3"/>
       <c r="AY63" s="3"/>
     </row>
-    <row r="64" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A64" s="23" t="s">
         <v>59</v>
       </c>
@@ -14130,7 +14130,7 @@
       <c r="AX64" s="3"/>
       <c r="AY64" s="3"/>
     </row>
-    <row r="65" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A65" s="23" t="s">
         <v>444</v>
       </c>
@@ -14187,7 +14187,7 @@
       <c r="AX65" s="3"/>
       <c r="AY65" s="3"/>
     </row>
-    <row r="66" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A66" s="23" t="s">
         <v>241</v>
       </c>
@@ -14244,7 +14244,7 @@
       <c r="AX66" s="3"/>
       <c r="AY66" s="3"/>
     </row>
-    <row r="67" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A67" s="23" t="s">
         <v>242</v>
       </c>
@@ -14307,7 +14307,7 @@
       <c r="AX67" s="3"/>
       <c r="AY67" s="3"/>
     </row>
-    <row r="68" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A68" s="23" t="s">
         <v>437</v>
       </c>
@@ -14441,7 +14441,7 @@
       <c r="AX69" s="3"/>
       <c r="AY69" s="3"/>
     </row>
-    <row r="70" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A70" s="23" t="s">
         <v>243</v>
       </c>
@@ -14506,7 +14506,7 @@
       <c r="AX70" s="3"/>
       <c r="AY70" s="3"/>
     </row>
-    <row r="71" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A71" s="23" t="s">
         <v>401</v>
       </c>
@@ -14565,7 +14565,7 @@
       <c r="AX71" s="3"/>
       <c r="AY71" s="3"/>
     </row>
-    <row r="72" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A72" s="23" t="s">
         <v>374</v>
       </c>
@@ -14630,7 +14630,7 @@
       <c r="AX72" s="3"/>
       <c r="AY72" s="3"/>
     </row>
-    <row r="73" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A73" s="23" t="s">
         <v>440</v>
       </c>
@@ -14752,7 +14752,7 @@
       <c r="AX74" s="3"/>
       <c r="AY74" s="3"/>
     </row>
-    <row r="75" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A75" s="23" t="s">
         <v>245</v>
       </c>
@@ -14809,7 +14809,7 @@
       <c r="AX75" s="3"/>
       <c r="AY75" s="3"/>
     </row>
-    <row r="76" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A76" s="23" t="s">
         <v>61</v>
       </c>
@@ -14878,7 +14878,7 @@
       <c r="AX76" s="3"/>
       <c r="AY76" s="3"/>
     </row>
-    <row r="77" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A77" s="23" t="s">
         <v>246</v>
       </c>
@@ -14943,7 +14943,7 @@
       <c r="AX77" s="3"/>
       <c r="AY77" s="3"/>
     </row>
-    <row r="78" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A78" s="23" t="s">
         <v>419</v>
       </c>
@@ -15061,7 +15061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A80" s="23" t="s">
         <v>451</v>
       </c>
@@ -15118,7 +15118,7 @@
       <c r="AX80" s="3"/>
       <c r="AY80" s="3"/>
     </row>
-    <row r="81" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A81" s="23" t="s">
         <v>412</v>
       </c>
@@ -15179,7 +15179,7 @@
       <c r="AX81" s="3"/>
       <c r="AY81" s="3"/>
     </row>
-    <row r="82" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A82" s="23" t="s">
         <v>62</v>
       </c>
@@ -15244,7 +15244,7 @@
       <c r="AX82" s="3"/>
       <c r="AY82" s="3"/>
     </row>
-    <row r="83" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A83" s="23" t="s">
         <v>386</v>
       </c>
@@ -15301,7 +15301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A84" s="23" t="s">
         <v>248</v>
       </c>
@@ -15439,7 +15439,7 @@
       <c r="AX85" s="3"/>
       <c r="AY85" s="3"/>
     </row>
-    <row r="86" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A86" s="23" t="s">
         <v>64</v>
       </c>
@@ -15516,7 +15516,7 @@
       <c r="AX86" s="3"/>
       <c r="AY86" s="3"/>
     </row>
-    <row r="87" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A87" s="23" t="s">
         <v>249</v>
       </c>
@@ -15577,7 +15577,7 @@
       <c r="AX87" s="3"/>
       <c r="AY87" s="3"/>
     </row>
-    <row r="88" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A88" s="23" t="s">
         <v>65</v>
       </c>
@@ -15640,7 +15640,7 @@
       <c r="AX88" s="3"/>
       <c r="AY88" s="3"/>
     </row>
-    <row r="89" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A89" s="23" t="s">
         <v>454</v>
       </c>
@@ -15697,7 +15697,7 @@
       <c r="AX89" s="3"/>
       <c r="AY89" s="3"/>
     </row>
-    <row r="90" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A90" s="23" t="s">
         <v>66</v>
       </c>
@@ -15821,7 +15821,7 @@
       <c r="AX91" s="3"/>
       <c r="AY91" s="3"/>
     </row>
-    <row r="92" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A92" s="23" t="s">
         <v>446</v>
       </c>
@@ -15937,7 +15937,7 @@
       <c r="AX93" s="3"/>
       <c r="AY93" s="3"/>
     </row>
-    <row r="94" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A94" s="23" t="s">
         <v>252</v>
       </c>
@@ -15998,7 +15998,7 @@
       <c r="AX94" s="3"/>
       <c r="AY94" s="3"/>
     </row>
-    <row r="95" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A95" s="23" t="s">
         <v>67</v>
       </c>
@@ -16126,7 +16126,7 @@
       <c r="AX96" s="3"/>
       <c r="AY96" s="3"/>
     </row>
-    <row r="97" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A97" s="23" t="s">
         <v>254</v>
       </c>
@@ -16187,7 +16187,7 @@
       <c r="AX97" s="3"/>
       <c r="AY97" s="3"/>
     </row>
-    <row r="98" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A98" s="23" t="s">
         <v>413</v>
       </c>
@@ -16244,7 +16244,7 @@
       <c r="AX98" s="3"/>
       <c r="AY98" s="3"/>
     </row>
-    <row r="99" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A99" s="23" t="s">
         <v>436</v>
       </c>
@@ -16362,7 +16362,7 @@
       <c r="AX100" s="3"/>
       <c r="AY100" s="3"/>
     </row>
-    <row r="101" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A101" s="23" t="s">
         <v>68</v>
       </c>
@@ -16437,7 +16437,7 @@
       <c r="AX101" s="3"/>
       <c r="AY101" s="3"/>
     </row>
-    <row r="102" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A102" s="23" t="s">
         <v>69</v>
       </c>
@@ -16563,7 +16563,7 @@
       <c r="AX103" s="3"/>
       <c r="AY103" s="3"/>
     </row>
-    <row r="104" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A104" s="23" t="s">
         <v>70</v>
       </c>
@@ -16689,7 +16689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A106" s="23" t="s">
         <v>458</v>
       </c>
@@ -16748,7 +16748,7 @@
       <c r="AX106" s="3"/>
       <c r="AY106" s="3"/>
     </row>
-    <row r="107" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A107" s="23" t="s">
         <v>441</v>
       </c>
@@ -16807,7 +16807,7 @@
       <c r="AX107" s="3"/>
       <c r="AY107" s="3"/>
     </row>
-    <row r="108" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A108" s="23" t="s">
         <v>430</v>
       </c>
@@ -16864,7 +16864,7 @@
       <c r="AX108" s="3"/>
       <c r="AY108" s="3"/>
     </row>
-    <row r="109" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A109" s="23" t="s">
         <v>71</v>
       </c>
@@ -16925,7 +16925,7 @@
       <c r="AX109" s="3"/>
       <c r="AY109" s="3"/>
     </row>
-    <row r="110" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A110" s="23" t="s">
         <v>72</v>
       </c>
@@ -16988,7 +16988,7 @@
       <c r="AX110" s="3"/>
       <c r="AY110" s="3"/>
     </row>
-    <row r="111" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A111" s="23" t="s">
         <v>466</v>
       </c>
@@ -17104,7 +17104,7 @@
       <c r="AX112" s="3"/>
       <c r="AY112" s="3"/>
     </row>
-    <row r="113" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A113" s="23" t="s">
         <v>455</v>
       </c>
@@ -17163,7 +17163,7 @@
       <c r="AX113" s="3"/>
       <c r="AY113" s="3"/>
     </row>
-    <row r="114" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A114" s="23" t="s">
         <v>258</v>
       </c>
@@ -17222,7 +17222,7 @@
       <c r="AX114" s="3"/>
       <c r="AY114" s="3"/>
     </row>
-    <row r="115" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A115" s="23" t="s">
         <v>445</v>
       </c>
@@ -17283,7 +17283,7 @@
       <c r="AX115" s="3"/>
       <c r="AY115" s="3"/>
     </row>
-    <row r="116" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A116" s="23" t="s">
         <v>73</v>
       </c>
@@ -17350,7 +17350,7 @@
       <c r="AX116" s="3"/>
       <c r="AY116" s="3"/>
     </row>
-    <row r="117" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A117" s="23" t="s">
         <v>259</v>
       </c>
@@ -17413,7 +17413,7 @@
       <c r="AX117" s="3"/>
       <c r="AY117" s="3"/>
     </row>
-    <row r="118" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A118" s="23" t="s">
         <v>74</v>
       </c>
@@ -17478,7 +17478,7 @@
       <c r="AX118" s="3"/>
       <c r="AY118" s="3"/>
     </row>
-    <row r="119" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A119" s="23" t="s">
         <v>260</v>
       </c>
@@ -17539,7 +17539,7 @@
       <c r="AX119" s="3"/>
       <c r="AY119" s="3"/>
     </row>
-    <row r="120" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A120" s="23" t="s">
         <v>387</v>
       </c>
@@ -17596,7 +17596,7 @@
       <c r="AX120" s="3"/>
       <c r="AY120" s="3"/>
     </row>
-    <row r="121" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A121" s="23" t="s">
         <v>75</v>
       </c>
@@ -17665,7 +17665,7 @@
       <c r="AX121" s="3"/>
       <c r="AY121" s="3"/>
     </row>
-    <row r="122" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A122" s="23" t="s">
         <v>261</v>
       </c>
@@ -17785,7 +17785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A124" s="23" t="s">
         <v>376</v>
       </c>
@@ -17842,7 +17842,7 @@
       <c r="AX124" s="3"/>
       <c r="AY124" s="3"/>
     </row>
-    <row r="125" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A125" s="23" t="s">
         <v>263</v>
       </c>
@@ -17903,7 +17903,7 @@
       <c r="AX125" s="3"/>
       <c r="AY125" s="3"/>
     </row>
-    <row r="126" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A126" s="23" t="s">
         <v>264</v>
       </c>
@@ -18106,7 +18106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A129" s="23" t="s">
         <v>77</v>
       </c>
@@ -18175,7 +18175,7 @@
       <c r="AX129" s="3"/>
       <c r="AY129" s="3"/>
     </row>
-    <row r="130" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A130" s="23" t="s">
         <v>78</v>
       </c>
@@ -18244,7 +18244,7 @@
       <c r="AX130" s="3"/>
       <c r="AY130" s="3"/>
     </row>
-    <row r="131" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A131" s="23" t="s">
         <v>410</v>
       </c>
@@ -18301,7 +18301,7 @@
       <c r="AX131" s="3"/>
       <c r="AY131" s="3"/>
     </row>
-    <row r="132" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A132" s="23" t="s">
         <v>266</v>
       </c>
@@ -18429,7 +18429,7 @@
       <c r="AX133" s="3"/>
       <c r="AY133" s="3"/>
     </row>
-    <row r="134" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A134" s="23" t="s">
         <v>79</v>
       </c>
@@ -18504,7 +18504,7 @@
       <c r="AX134" s="3"/>
       <c r="AY134" s="3"/>
     </row>
-    <row r="135" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A135" s="23" t="s">
         <v>380</v>
       </c>
@@ -18561,7 +18561,7 @@
       <c r="AX135" s="3"/>
       <c r="AY135" s="3"/>
     </row>
-    <row r="136" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A136" s="23" t="s">
         <v>80</v>
       </c>
@@ -18636,7 +18636,7 @@
       <c r="AX136" s="3"/>
       <c r="AY136" s="3"/>
     </row>
-    <row r="137" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A137" s="23" t="s">
         <v>81</v>
       </c>
@@ -18703,7 +18703,7 @@
       <c r="AX137" s="3"/>
       <c r="AY137" s="3"/>
     </row>
-    <row r="138" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A138" s="23" t="s">
         <v>268</v>
       </c>
@@ -18772,7 +18772,7 @@
       <c r="AX138" s="3"/>
       <c r="AY138" s="3"/>
     </row>
-    <row r="139" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A139" s="23" t="s">
         <v>82</v>
       </c>
@@ -18839,7 +18839,7 @@
       <c r="AX139" s="3"/>
       <c r="AY139" s="3"/>
     </row>
-    <row r="140" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A140" s="23" t="s">
         <v>269</v>
       </c>
@@ -18906,7 +18906,7 @@
       <c r="AX140" s="3"/>
       <c r="AY140" s="3"/>
     </row>
-    <row r="141" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A141" s="23" t="s">
         <v>270</v>
       </c>
@@ -18973,7 +18973,7 @@
       <c r="AX141" s="3"/>
       <c r="AY141" s="3"/>
     </row>
-    <row r="142" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A142" s="23" t="s">
         <v>432</v>
       </c>
@@ -19091,7 +19091,7 @@
       <c r="AX143" s="3"/>
       <c r="AY143" s="3"/>
     </row>
-    <row r="144" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A144" s="23" t="s">
         <v>84</v>
       </c>
@@ -19156,7 +19156,7 @@
       <c r="AX144" s="3"/>
       <c r="AY144" s="3"/>
     </row>
-    <row r="145" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A145" s="23" t="s">
         <v>377</v>
       </c>
@@ -19276,7 +19276,7 @@
       <c r="AX146" s="3"/>
       <c r="AY146" s="3"/>
     </row>
-    <row r="147" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A147" s="23" t="s">
         <v>428</v>
       </c>
@@ -19333,7 +19333,7 @@
       <c r="AX147" s="3"/>
       <c r="AY147" s="3"/>
     </row>
-    <row r="148" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A148" s="23" t="s">
         <v>388</v>
       </c>
@@ -19455,7 +19455,7 @@
       <c r="AX149" s="3"/>
       <c r="AY149" s="3"/>
     </row>
-    <row r="150" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A150" s="23" t="s">
         <v>274</v>
       </c>
@@ -19514,7 +19514,7 @@
       <c r="AX150" s="3"/>
       <c r="AY150" s="3"/>
     </row>
-    <row r="151" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A151" s="23" t="s">
         <v>275</v>
       </c>
@@ -19575,7 +19575,7 @@
       <c r="AX151" s="3"/>
       <c r="AY151" s="3"/>
     </row>
-    <row r="152" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A152" s="23" t="s">
         <v>85</v>
       </c>
@@ -19634,7 +19634,7 @@
       <c r="AX152" s="3"/>
       <c r="AY152" s="3"/>
     </row>
-    <row r="153" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A153" s="23" t="s">
         <v>276</v>
       </c>
@@ -19695,7 +19695,7 @@
       <c r="AX153" s="3"/>
       <c r="AY153" s="3"/>
     </row>
-    <row r="154" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A154" s="23" t="s">
         <v>87</v>
       </c>
@@ -19833,7 +19833,7 @@
       <c r="AX155" s="3"/>
       <c r="AY155" s="3"/>
     </row>
-    <row r="156" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A156" s="23" t="s">
         <v>277</v>
       </c>
@@ -19953,7 +19953,7 @@
       <c r="AX157" s="3"/>
       <c r="AY157" s="3"/>
     </row>
-    <row r="158" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A158" s="23" t="s">
         <v>279</v>
       </c>
@@ -20010,7 +20010,7 @@
       <c r="AX158" s="3"/>
       <c r="AY158" s="3"/>
     </row>
-    <row r="159" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A159" s="23" t="s">
         <v>89</v>
       </c>
@@ -20073,7 +20073,7 @@
       <c r="AX159" s="3"/>
       <c r="AY159" s="3"/>
     </row>
-    <row r="160" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A160" s="23" t="s">
         <v>90</v>
       </c>
@@ -20144,7 +20144,7 @@
       <c r="AX160" s="3"/>
       <c r="AY160" s="3"/>
     </row>
-    <row r="161" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A161" s="23" t="s">
         <v>417</v>
       </c>
@@ -20268,7 +20268,7 @@
       <c r="AX162" s="3"/>
       <c r="AY162" s="3"/>
     </row>
-    <row r="163" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A163" s="23" t="s">
         <v>281</v>
       </c>
@@ -20327,7 +20327,7 @@
       <c r="AX163" s="3"/>
       <c r="AY163" s="3"/>
     </row>
-    <row r="164" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A164" s="23" t="s">
         <v>282</v>
       </c>
@@ -20390,7 +20390,7 @@
       <c r="AX164" s="3"/>
       <c r="AY164" s="3"/>
     </row>
-    <row r="165" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A165" s="23" t="s">
         <v>283</v>
       </c>
@@ -20449,7 +20449,7 @@
       <c r="AX165" s="3"/>
       <c r="AY165" s="3"/>
     </row>
-    <row r="166" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A166" s="23" t="s">
         <v>91</v>
       </c>
@@ -20520,7 +20520,7 @@
       <c r="AX166" s="3"/>
       <c r="AY166" s="3"/>
     </row>
-    <row r="167" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A167" s="23" t="s">
         <v>464</v>
       </c>
@@ -20577,7 +20577,7 @@
       <c r="AX167" s="3"/>
       <c r="AY167" s="3"/>
     </row>
-    <row r="168" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A168" s="23" t="s">
         <v>284</v>
       </c>
@@ -20634,7 +20634,7 @@
       <c r="AX168" s="3"/>
       <c r="AY168" s="3"/>
     </row>
-    <row r="169" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A169" s="23" t="s">
         <v>92</v>
       </c>
@@ -20695,7 +20695,7 @@
       <c r="AX169" s="3"/>
       <c r="AY169" s="3"/>
     </row>
-    <row r="170" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A170" s="23" t="s">
         <v>94</v>
       </c>
@@ -20823,7 +20823,7 @@
       <c r="AX171" s="3"/>
       <c r="AY171" s="3"/>
     </row>
-    <row r="172" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A172" s="23" t="s">
         <v>96</v>
       </c>
@@ -20886,7 +20886,7 @@
       <c r="AX172" s="3"/>
       <c r="AY172" s="3"/>
     </row>
-    <row r="173" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A173" s="23" t="s">
         <v>97</v>
       </c>
@@ -20961,7 +20961,7 @@
       <c r="AX173" s="3"/>
       <c r="AY173" s="3"/>
     </row>
-    <row r="174" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A174" s="23" t="s">
         <v>98</v>
       </c>
@@ -21036,7 +21036,7 @@
       <c r="AX174" s="3"/>
       <c r="AY174" s="3"/>
     </row>
-    <row r="175" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A175" s="23" t="s">
         <v>99</v>
       </c>
@@ -21119,7 +21119,7 @@
       <c r="AX175" s="3"/>
       <c r="AY175" s="3"/>
     </row>
-    <row r="176" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A176" s="23" t="s">
         <v>100</v>
       </c>
@@ -21186,7 +21186,7 @@
       <c r="AX176" s="3"/>
       <c r="AY176" s="3"/>
     </row>
-    <row r="177" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A177" s="23" t="s">
         <v>384</v>
       </c>
@@ -21245,7 +21245,7 @@
       <c r="AX177" s="3"/>
       <c r="AY177" s="3"/>
     </row>
-    <row r="178" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A178" s="23" t="s">
         <v>101</v>
       </c>
@@ -21314,7 +21314,7 @@
       <c r="AX178" s="3"/>
       <c r="AY178" s="3"/>
     </row>
-    <row r="179" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A179" s="23" t="s">
         <v>433</v>
       </c>
@@ -21373,7 +21373,7 @@
       <c r="AX179" s="3"/>
       <c r="AY179" s="3"/>
     </row>
-    <row r="180" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A180" s="23" t="s">
         <v>378</v>
       </c>
@@ -21432,7 +21432,7 @@
       <c r="AX180" s="3"/>
       <c r="AY180" s="3"/>
     </row>
-    <row r="181" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A181" s="23" t="s">
         <v>285</v>
       </c>
@@ -21493,7 +21493,7 @@
       <c r="AX181" s="3"/>
       <c r="AY181" s="3"/>
     </row>
-    <row r="182" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A182" s="23" t="s">
         <v>102</v>
       </c>
@@ -21554,7 +21554,7 @@
       <c r="AX182" s="3"/>
       <c r="AY182" s="3"/>
     </row>
-    <row r="183" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A183" s="23" t="s">
         <v>104</v>
       </c>
@@ -21615,7 +21615,7 @@
       <c r="AX183" s="3"/>
       <c r="AY183" s="3"/>
     </row>
-    <row r="184" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A184" s="23" t="s">
         <v>105</v>
       </c>
@@ -21802,7 +21802,7 @@
       <c r="AX186" s="3"/>
       <c r="AY186" s="3"/>
     </row>
-    <row r="187" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A187" s="23" t="s">
         <v>457</v>
       </c>
@@ -21859,7 +21859,7 @@
       <c r="AX187" s="3"/>
       <c r="AY187" s="3"/>
     </row>
-    <row r="188" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A188" s="23" t="s">
         <v>107</v>
       </c>
@@ -21928,7 +21928,7 @@
       <c r="AX188" s="3"/>
       <c r="AY188" s="3"/>
     </row>
-    <row r="189" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A189" s="23" t="s">
         <v>287</v>
       </c>
@@ -21985,7 +21985,7 @@
       <c r="AX189" s="3"/>
       <c r="AY189" s="3"/>
     </row>
-    <row r="190" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A190" s="23" t="s">
         <v>288</v>
       </c>
@@ -22050,7 +22050,7 @@
       <c r="AX190" s="3"/>
       <c r="AY190" s="3"/>
     </row>
-    <row r="191" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A191" s="23" t="s">
         <v>108</v>
       </c>
@@ -22111,7 +22111,7 @@
       <c r="AX191" s="3"/>
       <c r="AY191" s="3"/>
     </row>
-    <row r="192" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A192" s="23" t="s">
         <v>415</v>
       </c>
@@ -22168,7 +22168,7 @@
       <c r="AX192" s="3"/>
       <c r="AY192" s="3"/>
     </row>
-    <row r="193" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A193" s="23" t="s">
         <v>422</v>
       </c>
@@ -22225,7 +22225,7 @@
       <c r="AX193" s="3"/>
       <c r="AY193" s="3"/>
     </row>
-    <row r="194" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A194" s="23" t="s">
         <v>109</v>
       </c>
@@ -22288,7 +22288,7 @@
       <c r="AX194" s="3"/>
       <c r="AY194" s="3"/>
     </row>
-    <row r="195" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A195" s="23" t="s">
         <v>110</v>
       </c>
@@ -22363,7 +22363,7 @@
       <c r="AX195" s="3"/>
       <c r="AY195" s="3"/>
     </row>
-    <row r="196" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A196" s="22" t="s">
         <v>111</v>
       </c>
@@ -22558,7 +22558,7 @@
       <c r="AX198" s="3"/>
       <c r="AY198" s="3"/>
     </row>
-    <row r="199" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A199" s="22" t="s">
         <v>447</v>
       </c>
@@ -22615,7 +22615,7 @@
       <c r="AX199" s="3"/>
       <c r="AY199" s="3"/>
     </row>
-    <row r="200" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A200" s="22" t="s">
         <v>113</v>
       </c>
@@ -22682,7 +22682,7 @@
       <c r="AX200" s="3"/>
       <c r="AY200" s="3"/>
     </row>
-    <row r="201" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A201" s="22" t="s">
         <v>114</v>
       </c>
@@ -22751,7 +22751,7 @@
       <c r="AX201" s="3"/>
       <c r="AY201" s="3"/>
     </row>
-    <row r="202" spans="1:204" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:204" ht="13" x14ac:dyDescent="0.3">
       <c r="A202" s="22" t="s">
         <v>404</v>
       </c>
@@ -23042,7 +23042,7 @@
       <c r="GU203" s="1"/>
       <c r="GV203" s="1"/>
     </row>
-    <row r="204" spans="1:204" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:204" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A204" s="22" t="s">
         <v>400</v>
       </c>
@@ -23254,7 +23254,7 @@
       <c r="GU204" s="1"/>
       <c r="GV204" s="1"/>
     </row>
-    <row r="205" spans="1:204" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:204" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A205" s="22" t="s">
         <v>461</v>
       </c>
@@ -23464,7 +23464,7 @@
       <c r="GU205" s="1"/>
       <c r="GV205" s="1"/>
     </row>
-    <row r="206" spans="1:204" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:204" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A206" s="22" t="s">
         <v>116</v>
       </c>
@@ -23900,7 +23900,7 @@
       <c r="GU207" s="1"/>
       <c r="GV207" s="1"/>
     </row>
-    <row r="208" spans="1:204" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:204" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A208" s="22" t="s">
         <v>424</v>
       </c>
@@ -24328,7 +24328,7 @@
       <c r="GU209" s="1"/>
       <c r="GV209" s="1"/>
     </row>
-    <row r="210" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A210" s="22" t="s">
         <v>117</v>
       </c>
@@ -24996,7 +24996,7 @@
       <c r="GW212" s="1"/>
       <c r="GX212" s="1"/>
     </row>
-    <row r="213" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A213" s="22" t="s">
         <v>294</v>
       </c>
@@ -25212,7 +25212,7 @@
       <c r="GW213" s="1"/>
       <c r="GX213" s="1"/>
     </row>
-    <row r="214" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A214" s="22" t="s">
         <v>295</v>
       </c>
@@ -25428,7 +25428,7 @@
       <c r="GW214" s="1"/>
       <c r="GX214" s="1"/>
     </row>
-    <row r="215" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A215" s="22" t="s">
         <v>296</v>
       </c>
@@ -25640,7 +25640,7 @@
       <c r="GW215" s="1"/>
       <c r="GX215" s="1"/>
     </row>
-    <row r="216" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A216" s="22" t="s">
         <v>459</v>
       </c>
@@ -25854,7 +25854,7 @@
       <c r="GW216" s="1"/>
       <c r="GX216" s="1"/>
     </row>
-    <row r="217" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A217" s="22" t="s">
         <v>456</v>
       </c>
@@ -26066,7 +26066,7 @@
       <c r="GW217" s="1"/>
       <c r="GX217" s="1"/>
     </row>
-    <row r="218" spans="1:206" s="4" customFormat="1" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:206" s="4" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A218" s="22" t="s">
         <v>297</v>
       </c>
@@ -26514,7 +26514,7 @@
       <c r="GW219" s="1"/>
       <c r="GX219" s="1"/>
     </row>
-    <row r="220" spans="1:206" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:206" ht="13" x14ac:dyDescent="0.3">
       <c r="A220" s="22" t="s">
         <v>299</v>
       </c>
@@ -26581,7 +26581,7 @@
       <c r="AX220" s="3"/>
       <c r="AY220" s="3"/>
     </row>
-    <row r="221" spans="1:206" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:206" ht="13" x14ac:dyDescent="0.3">
       <c r="A221" s="22" t="s">
         <v>300</v>
       </c>
@@ -26638,7 +26638,7 @@
       <c r="AX221" s="3"/>
       <c r="AY221" s="3"/>
     </row>
-    <row r="222" spans="1:206" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:206" ht="13" x14ac:dyDescent="0.3">
       <c r="A222" s="23" t="s">
         <v>120</v>
       </c>
@@ -26705,7 +26705,7 @@
       <c r="AX222" s="20"/>
       <c r="AY222" s="20"/>
     </row>
-    <row r="223" spans="1:206" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:206" ht="13" x14ac:dyDescent="0.3">
       <c r="A223" s="22" t="s">
         <v>301</v>
       </c>
@@ -26886,7 +26886,7 @@
       <c r="AX225" s="3"/>
       <c r="AY225" s="3"/>
     </row>
-    <row r="226" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A226" s="22" t="s">
         <v>303</v>
       </c>
@@ -26949,7 +26949,7 @@
       <c r="AX226" s="3"/>
       <c r="AY226" s="3"/>
     </row>
-    <row r="227" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A227" s="22" t="s">
         <v>304</v>
       </c>
@@ -27010,7 +27010,7 @@
       <c r="AX227" s="3"/>
       <c r="AY227" s="3"/>
     </row>
-    <row r="228" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A228" s="22" t="s">
         <v>305</v>
       </c>
@@ -27067,7 +27067,7 @@
       <c r="AX228" s="3"/>
       <c r="AY228" s="3"/>
     </row>
-    <row r="229" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A229" s="22" t="s">
         <v>123</v>
       </c>
@@ -27215,7 +27215,7 @@
       <c r="AX230" s="3"/>
       <c r="AY230" s="3"/>
     </row>
-    <row r="231" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A231" s="22" t="s">
         <v>408</v>
       </c>
@@ -27383,7 +27383,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A233" s="22" t="s">
         <v>125</v>
       </c>
@@ -27513,7 +27513,7 @@
       <c r="AX234" s="3"/>
       <c r="AY234" s="3"/>
     </row>
-    <row r="235" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A235" s="22" t="s">
         <v>434</v>
       </c>
@@ -27629,7 +27629,7 @@
       <c r="AX236" s="3"/>
       <c r="AY236" s="3"/>
     </row>
-    <row r="237" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A237" s="22" t="s">
         <v>308</v>
       </c>
@@ -27696,7 +27696,7 @@
       <c r="AX237" s="3"/>
       <c r="AY237" s="3"/>
     </row>
-    <row r="238" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A238" s="22" t="s">
         <v>309</v>
       </c>
@@ -27755,7 +27755,7 @@
       <c r="AX238" s="3"/>
       <c r="AY238" s="3"/>
     </row>
-    <row r="239" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A239" s="22" t="s">
         <v>310</v>
       </c>
@@ -27889,7 +27889,7 @@
       <c r="AX240" s="3"/>
       <c r="AY240" s="3"/>
     </row>
-    <row r="241" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A241" s="22" t="s">
         <v>448</v>
       </c>
@@ -28153,7 +28153,7 @@
       <c r="AX244" s="3"/>
       <c r="AY244" s="3"/>
     </row>
-    <row r="245" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A245" s="22" t="s">
         <v>314</v>
       </c>
@@ -28340,7 +28340,7 @@
       <c r="AX247" s="3"/>
       <c r="AY247" s="3"/>
     </row>
-    <row r="248" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A248" s="22" t="s">
         <v>316</v>
       </c>
@@ -28403,7 +28403,7 @@
       <c r="AX248" s="3"/>
       <c r="AY248" s="3"/>
     </row>
-    <row r="249" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A249" s="22" t="s">
         <v>130</v>
       </c>
@@ -28480,7 +28480,7 @@
       <c r="AX249" s="3"/>
       <c r="AY249" s="3"/>
     </row>
-    <row r="250" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A250" s="23" t="s">
         <v>317</v>
       </c>
@@ -28543,7 +28543,7 @@
       <c r="AX250" s="20"/>
       <c r="AY250" s="20"/>
     </row>
-    <row r="251" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A251" s="22" t="s">
         <v>403</v>
       </c>
@@ -28659,7 +28659,7 @@
       <c r="AX252" s="3"/>
       <c r="AY252" s="3"/>
     </row>
-    <row r="253" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A253" s="22" t="s">
         <v>318</v>
       </c>
@@ -28789,7 +28789,7 @@
       <c r="AX254" s="3"/>
       <c r="AY254" s="3"/>
     </row>
-    <row r="255" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A255" s="22" t="s">
         <v>421</v>
       </c>
@@ -28984,7 +28984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="258" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A258" s="22" t="s">
         <v>391</v>
       </c>
@@ -29041,7 +29041,7 @@
       <c r="AX258" s="3"/>
       <c r="AY258" s="3"/>
     </row>
-    <row r="259" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A259" s="22" t="s">
         <v>133</v>
       </c>
@@ -29108,7 +29108,7 @@
       <c r="AX259" s="3"/>
       <c r="AY259" s="3"/>
     </row>
-    <row r="260" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A260" s="22" t="s">
         <v>134</v>
       </c>
@@ -29230,7 +29230,7 @@
       <c r="AX261" s="3"/>
       <c r="AY261" s="3"/>
     </row>
-    <row r="262" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A262" s="22" t="s">
         <v>463</v>
       </c>
@@ -29287,7 +29287,7 @@
       <c r="AX262" s="3"/>
       <c r="AY262" s="3"/>
     </row>
-    <row r="263" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A263" s="22" t="s">
         <v>407</v>
       </c>
@@ -29344,7 +29344,7 @@
       <c r="AX263" s="3"/>
       <c r="AY263" s="3"/>
     </row>
-    <row r="264" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A264" s="22" t="s">
         <v>135</v>
       </c>
@@ -29411,7 +29411,7 @@
       <c r="AX264" s="3"/>
       <c r="AY264" s="3"/>
     </row>
-    <row r="265" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A265" s="22" t="s">
         <v>462</v>
       </c>
@@ -29468,7 +29468,7 @@
       <c r="AX265" s="3"/>
       <c r="AY265" s="3"/>
     </row>
-    <row r="266" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A266" s="22" t="s">
         <v>322</v>
       </c>
@@ -29525,7 +29525,7 @@
       <c r="AX266" s="3"/>
       <c r="AY266" s="3"/>
     </row>
-    <row r="267" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A267" s="22" t="s">
         <v>323</v>
       </c>
@@ -29582,7 +29582,7 @@
       <c r="AX267" s="3"/>
       <c r="AY267" s="3"/>
     </row>
-    <row r="268" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A268" s="22" t="s">
         <v>420</v>
       </c>
@@ -29639,7 +29639,7 @@
       <c r="AX268" s="3"/>
       <c r="AY268" s="3"/>
     </row>
-    <row r="269" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A269" s="22" t="s">
         <v>324</v>
       </c>
@@ -29828,7 +29828,7 @@
       <c r="AX271" s="3"/>
       <c r="AY271" s="3"/>
     </row>
-    <row r="272" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A272" s="22" t="s">
         <v>137</v>
       </c>
@@ -29903,7 +29903,7 @@
       <c r="AX272" s="3"/>
       <c r="AY272" s="3"/>
     </row>
-    <row r="273" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A273" s="22" t="s">
         <v>138</v>
       </c>
@@ -29968,7 +29968,7 @@
       <c r="AX273" s="3"/>
       <c r="AY273" s="3"/>
     </row>
-    <row r="274" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A274" s="22" t="s">
         <v>139</v>
       </c>
@@ -30037,7 +30037,7 @@
       <c r="AX274" s="3"/>
       <c r="AY274" s="3"/>
     </row>
-    <row r="275" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A275" s="23" t="s">
         <v>140</v>
       </c>
@@ -30104,7 +30104,7 @@
       <c r="AX275" s="20"/>
       <c r="AY275" s="20"/>
     </row>
-    <row r="276" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A276" s="22" t="s">
         <v>141</v>
       </c>
@@ -30175,7 +30175,7 @@
       <c r="AX276" s="3"/>
       <c r="AY276" s="3"/>
     </row>
-    <row r="277" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A277" s="22" t="s">
         <v>326</v>
       </c>
@@ -30234,7 +30234,7 @@
       <c r="AX277" s="3"/>
       <c r="AY277" s="3"/>
     </row>
-    <row r="278" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A278" s="22" t="s">
         <v>327</v>
       </c>
@@ -30301,7 +30301,7 @@
       <c r="AX278" s="3"/>
       <c r="AY278" s="3"/>
     </row>
-    <row r="279" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A279" s="22" t="s">
         <v>142</v>
       </c>
@@ -30368,7 +30368,7 @@
       <c r="AX279" s="3"/>
       <c r="AY279" s="3"/>
     </row>
-    <row r="280" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A280" s="22" t="s">
         <v>143</v>
       </c>
@@ -30429,7 +30429,7 @@
       <c r="AX280" s="3"/>
       <c r="AY280" s="3"/>
     </row>
-    <row r="281" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A281" s="22" t="s">
         <v>389</v>
       </c>
@@ -30488,7 +30488,7 @@
       <c r="AX281" s="3"/>
       <c r="AY281" s="3"/>
     </row>
-    <row r="282" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A282" s="22" t="s">
         <v>328</v>
       </c>
@@ -30561,7 +30561,7 @@
       <c r="AX282" s="3"/>
       <c r="AY282" s="3"/>
     </row>
-    <row r="283" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A283" s="22" t="s">
         <v>329</v>
       </c>
@@ -30758,7 +30758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="286" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A286" s="22" t="s">
         <v>409</v>
       </c>
@@ -30815,7 +30815,7 @@
       <c r="AX286" s="3"/>
       <c r="AY286" s="3"/>
     </row>
-    <row r="287" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A287" s="22" t="s">
         <v>393</v>
       </c>
@@ -30874,7 +30874,7 @@
       <c r="AX287" s="3"/>
       <c r="AY287" s="3"/>
     </row>
-    <row r="288" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A288" s="22" t="s">
         <v>145</v>
       </c>
@@ -30943,7 +30943,7 @@
       <c r="AX288" s="3"/>
       <c r="AY288" s="3"/>
     </row>
-    <row r="289" spans="1:51" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A289" s="22" t="s">
         <v>465</v>
       </c>
@@ -31000,7 +31000,7 @@
       <c r="AX289" s="3"/>
       <c r="AY289" s="3"/>
     </row>
-    <row r="290" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A290" s="22" t="s">
         <v>146</v>
       </c>
@@ -31132,7 +31132,7 @@
       <c r="AX291" s="3"/>
       <c r="AY291" s="3"/>
     </row>
-    <row r="292" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A292" s="22" t="s">
         <v>332</v>
       </c>
@@ -31260,7 +31260,7 @@
       <c r="AX293" s="3"/>
       <c r="AY293" s="3"/>
     </row>
-    <row r="294" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A294" s="22" t="s">
         <v>147</v>
       </c>
@@ -31329,7 +31329,7 @@
       <c r="AX294" s="3"/>
       <c r="AY294" s="3"/>
     </row>
-    <row r="295" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A295" s="22" t="s">
         <v>148</v>
       </c>
@@ -31400,7 +31400,7 @@
       <c r="AX295" s="3"/>
       <c r="AY295" s="3"/>
     </row>
-    <row r="296" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A296" s="22" t="s">
         <v>334</v>
       </c>
@@ -31457,7 +31457,7 @@
       <c r="AX296" s="3"/>
       <c r="AY296" s="3"/>
     </row>
-    <row r="297" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A297" s="22" t="s">
         <v>149</v>
       </c>
@@ -31520,7 +31520,7 @@
       <c r="AX297" s="3"/>
       <c r="AY297" s="3"/>
     </row>
-    <row r="298" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A298" s="22" t="s">
         <v>335</v>
       </c>
@@ -31577,7 +31577,7 @@
       <c r="AX298" s="3"/>
       <c r="AY298" s="3"/>
     </row>
-    <row r="299" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A299" s="22" t="s">
         <v>150</v>
       </c>
@@ -31644,7 +31644,7 @@
       <c r="AX299" s="3"/>
       <c r="AY299" s="3"/>
     </row>
-    <row r="300" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A300" s="22" t="s">
         <v>151</v>
       </c>
@@ -31705,7 +31705,7 @@
       <c r="AX300" s="3"/>
       <c r="AY300" s="3"/>
     </row>
-    <row r="301" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A301" s="22" t="s">
         <v>418</v>
       </c>
@@ -31764,7 +31764,7 @@
       <c r="AX301" s="3"/>
       <c r="AY301" s="3"/>
     </row>
-    <row r="302" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A302" s="22" t="s">
         <v>450</v>
       </c>
@@ -31821,7 +31821,7 @@
       <c r="AX302" s="3"/>
       <c r="AY302" s="3"/>
     </row>
-    <row r="303" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A303" s="22" t="s">
         <v>336</v>
       </c>
@@ -31878,7 +31878,7 @@
       <c r="AX303" s="3"/>
       <c r="AY303" s="3"/>
     </row>
-    <row r="304" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A304" s="22" t="s">
         <v>337</v>
       </c>
@@ -31937,7 +31937,7 @@
       <c r="AX304" s="3"/>
       <c r="AY304" s="3"/>
     </row>
-    <row r="305" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A305" s="22" t="s">
         <v>338</v>
       </c>
@@ -31996,7 +31996,7 @@
       <c r="AX305" s="3"/>
       <c r="AY305" s="3"/>
     </row>
-    <row r="306" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A306" s="23" t="s">
         <v>153</v>
       </c>
@@ -32069,7 +32069,7 @@
       <c r="AX306" s="20"/>
       <c r="AY306" s="20"/>
     </row>
-    <row r="307" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A307" s="22" t="s">
         <v>339</v>
       </c>
@@ -32128,7 +32128,7 @@
       <c r="AX307" s="3"/>
       <c r="AY307" s="3"/>
     </row>
-    <row r="308" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A308" s="22" t="s">
         <v>154</v>
       </c>
@@ -32203,7 +32203,7 @@
       <c r="AX308" s="3"/>
       <c r="AY308" s="3"/>
     </row>
-    <row r="309" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A309" s="22" t="s">
         <v>340</v>
       </c>
@@ -32262,7 +32262,7 @@
       <c r="AX309" s="3"/>
       <c r="AY309" s="3"/>
     </row>
-    <row r="310" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A310" s="22" t="s">
         <v>341</v>
       </c>
@@ -32321,7 +32321,7 @@
       <c r="AX310" s="3"/>
       <c r="AY310" s="3"/>
     </row>
-    <row r="311" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A311" s="22" t="s">
         <v>453</v>
       </c>
@@ -32439,7 +32439,7 @@
       <c r="AX312" s="3"/>
       <c r="AY312" s="3"/>
     </row>
-    <row r="313" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A313" s="22" t="s">
         <v>342</v>
       </c>
@@ -32496,7 +32496,7 @@
       <c r="AX313" s="3"/>
       <c r="AY313" s="3"/>
     </row>
-    <row r="314" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A314" s="22" t="s">
         <v>343</v>
       </c>
@@ -32689,7 +32689,7 @@
       <c r="AX316" s="3"/>
       <c r="AY316" s="3"/>
     </row>
-    <row r="317" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A317" s="22" t="s">
         <v>156</v>
       </c>
@@ -32987,7 +32987,7 @@
       <c r="AX320" s="3"/>
       <c r="AY320" s="3"/>
     </row>
-    <row r="321" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A321" s="22" t="s">
         <v>346</v>
       </c>
@@ -33186,7 +33186,7 @@
       <c r="AX323" s="3"/>
       <c r="AY323" s="3"/>
     </row>
-    <row r="324" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A324" s="22" t="s">
         <v>161</v>
       </c>
@@ -33255,7 +33255,7 @@
       <c r="AX324" s="3"/>
       <c r="AY324" s="3"/>
     </row>
-    <row r="325" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A325" s="22" t="s">
         <v>162</v>
       </c>
@@ -33322,7 +33322,7 @@
       <c r="AX325" s="3"/>
       <c r="AY325" s="3"/>
     </row>
-    <row r="326" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A326" s="22" t="s">
         <v>163</v>
       </c>
@@ -33397,7 +33397,7 @@
       <c r="AX326" s="3"/>
       <c r="AY326" s="3"/>
     </row>
-    <row r="327" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A327" s="22" t="s">
         <v>164</v>
       </c>
@@ -33462,7 +33462,7 @@
       <c r="AX327" s="3"/>
       <c r="AY327" s="3"/>
     </row>
-    <row r="328" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A328" s="22" t="s">
         <v>165</v>
       </c>
@@ -33529,7 +33529,7 @@
       <c r="AX328" s="3"/>
       <c r="AY328" s="3"/>
     </row>
-    <row r="329" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A329" s="22" t="s">
         <v>429</v>
       </c>
@@ -33588,7 +33588,7 @@
       <c r="AX329" s="3"/>
       <c r="AY329" s="3"/>
     </row>
-    <row r="330" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A330" s="22" t="s">
         <v>427</v>
       </c>
@@ -33704,7 +33704,7 @@
       <c r="AX331" s="3"/>
       <c r="AY331" s="3"/>
     </row>
-    <row r="332" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A332" s="22" t="s">
         <v>349</v>
       </c>
@@ -33761,7 +33761,7 @@
       <c r="AX332" s="3"/>
       <c r="AY332" s="3"/>
     </row>
-    <row r="333" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A333" s="22" t="s">
         <v>350</v>
       </c>
@@ -33883,7 +33883,7 @@
       <c r="AX334" s="3"/>
       <c r="AY334" s="3"/>
     </row>
-    <row r="335" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A335" s="22" t="s">
         <v>352</v>
       </c>
@@ -33940,7 +33940,7 @@
       <c r="AX335" s="3"/>
       <c r="AY335" s="3"/>
     </row>
-    <row r="336" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A336" s="22" t="s">
         <v>353</v>
       </c>
@@ -33997,7 +33997,7 @@
       <c r="AX336" s="3"/>
       <c r="AY336" s="3"/>
     </row>
-    <row r="337" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A337" s="22" t="s">
         <v>354</v>
       </c>
@@ -34058,7 +34058,7 @@
       <c r="AX337" s="3"/>
       <c r="AY337" s="3"/>
     </row>
-    <row r="338" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A338" s="22" t="s">
         <v>166</v>
       </c>
@@ -34135,7 +34135,7 @@
       <c r="AX338" s="3"/>
       <c r="AY338" s="3"/>
     </row>
-    <row r="339" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A339" s="22" t="s">
         <v>355</v>
       </c>
@@ -34200,7 +34200,7 @@
       <c r="AX339" s="3"/>
       <c r="AY339" s="3"/>
     </row>
-    <row r="340" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A340" s="22" t="s">
         <v>356</v>
       </c>
@@ -34257,7 +34257,7 @@
       <c r="AX340" s="3"/>
       <c r="AY340" s="3"/>
     </row>
-    <row r="341" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A341" s="22" t="s">
         <v>357</v>
       </c>
@@ -34387,7 +34387,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="343" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A343" s="22" t="s">
         <v>385</v>
       </c>
@@ -34649,7 +34649,7 @@
       <c r="AX346" s="3"/>
       <c r="AY346" s="3"/>
     </row>
-    <row r="347" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A347" s="22" t="s">
         <v>361</v>
       </c>
@@ -34714,7 +34714,7 @@
       <c r="AX347" s="3"/>
       <c r="AY347" s="3"/>
     </row>
-    <row r="348" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A348" s="22" t="s">
         <v>381</v>
       </c>
@@ -34771,7 +34771,7 @@
       <c r="AX348" s="3"/>
       <c r="AY348" s="3"/>
     </row>
-    <row r="349" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A349" s="22" t="s">
         <v>382</v>
       </c>
@@ -34828,7 +34828,7 @@
       <c r="AX349" s="3"/>
       <c r="AY349" s="3"/>
     </row>
-    <row r="350" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A350" s="22" t="s">
         <v>362</v>
       </c>
@@ -34891,7 +34891,7 @@
       <c r="AX350" s="3"/>
       <c r="AY350" s="3"/>
     </row>
-    <row r="351" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A351" s="22" t="s">
         <v>169</v>
       </c>
@@ -35033,7 +35033,7 @@
       <c r="AX352" s="3"/>
       <c r="AY352" s="3"/>
     </row>
-    <row r="353" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A353" s="22" t="s">
         <v>364</v>
       </c>
@@ -35090,7 +35090,7 @@
       <c r="AX353" s="3"/>
       <c r="AY353" s="3"/>
     </row>
-    <row r="354" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A354" s="22" t="s">
         <v>365</v>
       </c>
@@ -35151,7 +35151,7 @@
       <c r="AX354" s="3"/>
       <c r="AY354" s="3"/>
     </row>
-    <row r="355" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A355" s="22" t="s">
         <v>170</v>
       </c>
@@ -35220,7 +35220,7 @@
       <c r="AX355" s="3"/>
       <c r="AY355" s="3"/>
     </row>
-    <row r="356" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A356" s="22" t="s">
         <v>366</v>
       </c>
@@ -35340,7 +35340,7 @@
       <c r="AX357" s="3"/>
       <c r="AY357" s="3"/>
     </row>
-    <row r="358" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A358" s="22" t="s">
         <v>373</v>
       </c>
@@ -35399,7 +35399,7 @@
       <c r="AX358" s="3"/>
       <c r="AY358" s="3"/>
     </row>
-    <row r="359" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A359" s="22" t="s">
         <v>368</v>
       </c>
@@ -35466,7 +35466,7 @@
       <c r="AX359" s="3"/>
       <c r="AY359" s="3"/>
     </row>
-    <row r="360" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A360" s="22" t="s">
         <v>172</v>
       </c>
@@ -35527,7 +35527,7 @@
       <c r="AX360" s="3"/>
       <c r="AY360" s="3"/>
     </row>
-    <row r="361" spans="1:51" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A361" s="22" t="s">
         <v>173</v>
       </c>
@@ -35592,7 +35592,7 @@
       <c r="AX361" s="3"/>
       <c r="AY361" s="3"/>
     </row>
-    <row r="362" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A362" s="22" t="s">
         <v>174</v>
       </c>
@@ -35661,7 +35661,7 @@
       <c r="AX362" s="3"/>
       <c r="AY362" s="3"/>
     </row>
-    <row r="363" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A363" s="22" t="s">
         <v>449</v>
       </c>
@@ -35720,7 +35720,7 @@
       <c r="AX363" s="3"/>
       <c r="AY363" s="3"/>
     </row>
-    <row r="364" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A364" s="22" t="s">
         <v>369</v>
       </c>
@@ -35781,7 +35781,7 @@
       <c r="AX364" s="3"/>
       <c r="AY364" s="3"/>
     </row>
-    <row r="365" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A365" s="22" t="s">
         <v>423</v>
       </c>
@@ -35897,7 +35897,7 @@
       <c r="AX366" s="3"/>
       <c r="AY366" s="3"/>
     </row>
-    <row r="367" spans="1:51" ht="13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A367" s="22" t="s">
         <v>371</v>
       </c>
@@ -35964,7 +35964,6 @@
       <c r="AX367" s="3"/>
       <c r="AY367" s="3"/>
     </row>
-    <row r="368" spans="1:51" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="370" spans="1:52" ht="13" x14ac:dyDescent="0.3">
       <c r="B370" s="14"/>
       <c r="C370" s="14"/>
@@ -36071,7 +36070,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="393" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A393" s="26"/>
       <c r="B393" s="26"/>
       <c r="C393" s="26"/>
@@ -36124,7 +36123,7 @@
       <c r="AX393" s="26"/>
       <c r="AY393" s="26"/>
     </row>
-    <row r="394" spans="1:51" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:51" ht="13" x14ac:dyDescent="0.3">
       <c r="A394" s="26"/>
       <c r="B394" s="26"/>
       <c r="C394" s="26"/>

</xml_diff>